<commit_message>
Update program schedule for Endogineco 2026 with speaker changes and session details
- Replaced speaker names for specific sessions to reflect accurate information: Patrick Belilis is now Fabio Ohara for a session on nerve injuries, and added Guilherme Zanluchi as the speaker for a session on retained ovular remnants.
- Updated the symposium title to include the sponsor name "ZYDUS" for clarity.
- Enhanced the "CIRURGIAS AO VIVO" section with clearer formatting and additional details about participating hospitals and speakers.
- Adjusted session titles and descriptions for better clarity and organization in the schedule.
</commit_message>
<xml_diff>
--- a/endogineco2026/schedule/programacao-preliminar-2026.xlsx
+++ b/endogineco2026/schedule/programacao-preliminar-2026.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Programação CONGRESSO " sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Programação CONGRESSO '!$A$1:$C$124</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Programação CONGRESSO '!$A$1:$C$127</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="249">
   <si>
     <t xml:space="preserve"> CONGRESSO ENDOGINECO </t>
   </si>
@@ -93,7 +93,7 @@
     <t xml:space="preserve">Principais lesões nervosas na Endometriose ? Quais os principais sintomas ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Patrick Belilis - SP </t>
+    <t xml:space="preserve">Fabio Ohara - SP </t>
   </si>
   <si>
     <t xml:space="preserve">09:20 - 09:40
@@ -192,6 +192,9 @@
     <t xml:space="preserve">Os desafios da retenção de restos ovulares - Como a Histeroscopia pode ajudar? </t>
   </si>
   <si>
+    <t xml:space="preserve">Guilherme Zanluchi -SP</t>
+  </si>
+  <si>
     <t xml:space="preserve">11:30 - 11:40
 (10 min) 
 </t>
@@ -201,7 +204,23 @@
 (20 min)</t>
   </si>
   <si>
-    <t xml:space="preserve">SIMPÓSIO - A reposição de Ferro - Item fundamental para uma cirurgia segura </t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SIMPÓSIO ZYDUS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -  A reposição de Ferro - Item fundamental para uma cirurgia segura </t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Jardel Soares - PE </t>
@@ -222,7 +241,8 @@
 (2 horas) </t>
   </si>
   <si>
-    <t xml:space="preserve">CIRURGIAS AO VIVO                                                                                                                                              Presidente: Mauro Aguiar - PE
+    <t xml:space="preserve">CIRURGIAS AO VIVO                                                                                                                                            
+Presidente: Mauro Aguiar - PE
 Debatedores: Kelvin Manderson - PE , Neidson Menezes PE , Phabllo Rodrigo - PE </t>
   </si>
   <si>
@@ -316,9 +336,41 @@
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">* Hospital das nações CWB  
-Mônica Zomer PR 
-William Kondo PR</t>
+      <t xml:space="preserve">* Hospital das Nações CWB  
+Mônica Zomer PR -  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="2"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SALA 1</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="2" tint="-0.89999084444715716"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+William Kondo PR - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="2"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SALA 2</t>
     </r>
     <r>
       <rPr>
@@ -408,31 +460,15 @@
     <t xml:space="preserve">Andreisa Bilhar - CE</t>
   </si>
   <si>
+    <t xml:space="preserve">Conferências </t>
+  </si>
+  <si>
     <t xml:space="preserve">16:50 - 17:15
 (25 min) </t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Conferência - </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Como a IA pode influenciar  sua conduta do consultório ao pós- cirúrgico?</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t xml:space="preserve"> Como a IA pode influenciar  sua conduta do consultório ao pós- cirúrgico?
 Presidente: Edilberto Rocha - PE </t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">17:15 - 17:25
@@ -453,9 +489,26 @@
 Como ter um consultório de sucesso                                                                                                                        Coordenadora: Mariana Muniz</t>
   </si>
   <si>
-    <t xml:space="preserve">Rosaura Almeida - PE, Marcos Saturnino - PE, Isaura Vieira - DF
-Urologista 
-Kathyane Lustosa - CE, Mayara Macedo -PE, Pericles Oliveira - PB, Psicólogo </t>
+    <r>
+      <t xml:space="preserve">Rosaura Almeida - PE, nutri 
+Isaura Vieira - DF acupunturista
+Arthur Farias -PB urologista 
+Kathyane Lustosa - CE, Gineco
+Mayara Macedo -PE,Fisio pel
+Pericles Oliveira - PB, Procto 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="10"/>
+        <color indexed="2"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Macira Sotero- PE, Psicóloga </t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Cerimônia abertura </t>
@@ -469,9 +522,21 @@
 40 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">MESA 1 -  No meu consultório           
+    <r>
+      <t xml:space="preserve">MESA 1 -  No meu consultório           
 Presidente: Simone Carvalho - PE 
-Debatedores:</t>
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FFAC0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Debatedores:</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">08:25 - 08:45 
@@ -586,6 +651,9 @@
     <t xml:space="preserve">Como eu tratei essa lesão ureteral de endometriose </t>
   </si>
   <si>
+    <t xml:space="preserve">Vinícius Araújo - RJ </t>
+  </si>
+  <si>
     <t xml:space="preserve">11:35 - 11:55
 (20 min) </t>
   </si>
@@ -616,32 +684,60 @@
     <t xml:space="preserve">Mariana Vieira - SP</t>
   </si>
   <si>
-    <t xml:space="preserve">12:35 - 12:50
+    <t xml:space="preserve">12:35 - 13:30
+(55 min)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRURGIAS AO VIVO - NA SALA A                                                                                                                                             
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:00 - 16:15
 (15 min)</t>
   </si>
   <si>
-    <t xml:space="preserve">SIMPÓSIO  - A reposição de Ferro - Item fundamental para uma cirurgia segura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12:50 - 13:30
-(40 min)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRURGIAS AO VIVO                                                                                                                                              
-Presidente: Mauro Aguiar - PE
-Debatedores: Kelvin Manderson - PE , Neidson Menezes PE , Phabllo Rodrigo - PE </t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:00 - 17:10
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SIMPÓSIO PATROCINADO BAYER </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - Tratamento Clínico da Endometriose segundo o protocolo da ACOH 2026 </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">16:15 - 17:25
 (01 hora e 
 10 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">MESA 2 - Imagem        
-Presidente: Taciana Morais</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:00 - 16:30
+    <r>
+      <t xml:space="preserve">MESA 2 - Imagem        
+Presidente: Taciana Morais
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FFED0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Debatedores:</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">16:15 - 16:45
 (30 min) </t>
   </si>
   <si>
@@ -659,41 +755,27 @@
     <t xml:space="preserve">O que não pode faltar na ressonância para rastreio de endometriose ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Rafaela Agonis - BA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:30 - 16:45
-(15 min)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como a  reconstrução três D veio para trazer um  apoio ao cirurgião ? Te mostro na prática</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Italo Cruz - PE </t>
-  </si>
-  <si>
     <t xml:space="preserve">16:45 - 17:00
 (15 min)</t>
   </si>
   <si>
+    <t xml:space="preserve">Como a  reconstrução três D veio para trazer um  apoio ao cirurgião ? Te mostro na prática</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Italo Cruz - PE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:00 - 17:15
+(15 min)</t>
+  </si>
+  <si>
     <t xml:space="preserve">A IA substituirá o humano  no diagnóstico radiológico da endometriose?</t>
   </si>
   <si>
     <t xml:space="preserve">Nadja Rolim - PE </t>
   </si>
   <si>
-    <t xml:space="preserve">17:00 - 17:10
-(10 min) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:10 - 17:25
-(15 min)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIMPÓSIO PATROCINADO BAYER  - Tratamento Clínico da Endometriose segundo o protocolo da ACOH 2026 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:15 - 18:00
+    <t xml:space="preserve">17:25 - 18:10
 (45 min) </t>
   </si>
   <si>
@@ -706,7 +788,6 @@
         <b/>
         <i/>
         <sz val="10"/>
-        <color theme="1"/>
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
@@ -714,7 +795,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Caso Clínico 1 - TUMOR ANEXIAL </t>
+    <t xml:space="preserve">Caso Clínico 1 - Endometeiose severa com exclusão renal  </t>
   </si>
   <si>
     <t xml:space="preserve">Caso Clínico 2 - PROLAPSO + INCONTINÊNCIA URINÁRIA</t>
@@ -739,7 +820,7 @@
   </si>
   <si>
     <t xml:space="preserve">CIRURGIAS AO VIVO                                                                                                                                                                           Presidente : Iolanda Matias - PE 
-Debatedores: Gilvan Santos - PE, Mariana Roma - PE, Felipe Rocha - PE, Guilherme zanluchi SP</t>
+Debatedores:  Mariana Roma - PE, Felipe Rocha - PE, Guilherme Zanluchi - SP, Felipe Rocha - PB</t>
   </si>
   <si>
     <r>
@@ -806,7 +887,7 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">* Hospital Barão de Lucena  - PE
-Condução caso: Eveline Martins Sampaio - PE 
+Condução caso: Eveline Martins - PE 
 Sara Arcanjo - PE /
 Andreisa Bilhar - CE</t>
     </r>
@@ -843,7 +924,7 @@
       </rPr>
       <t xml:space="preserve">* Hospital Itaim Bibi - SP 
 Dr Paulo Ayroza /
-Helizabeth Salomão</t>
+Helizabeth Salomão </t>
     </r>
     <r>
       <rPr>
@@ -871,6 +952,10 @@
   <si>
     <t xml:space="preserve">10:00 - 10:30 
 (30 min) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conferências   
+ Presidente : Walter Ivo Paiva PE </t>
   </si>
   <si>
     <t xml:space="preserve">10:30 - 10:50         (20 min)</t>
@@ -956,9 +1041,21 @@
 10 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">MESA 1 - Infertilidade e Endometriose 
-Presidente:
+    <r>
+      <t xml:space="preserve">MESA 1 - Infertilidade e Endometriose 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FFAC0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Presidente:
 Debatedores:</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">11:25 - 11:40 
@@ -1006,7 +1103,11 @@
 (20 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">INTERVALO </t>
+    <t xml:space="preserve">SIMPÓSIO ABIACON - LUNCH BOX </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conferências   
+ Presidente : Jardel Soares - PE </t>
   </si>
   <si>
     <t xml:space="preserve">12:55 - 13:15
@@ -1067,10 +1168,31 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">MESA 2 - Coloproctologia no painel         
+    <r>
+      <t xml:space="preserve">MESA 2 - Coloproctologia no painel         
 Presidente : Marcos Saturnino - PE
-Debatedores:
 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FFAC0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Debatedores:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">13:35 - 14:05            (30 min)
@@ -1119,7 +1241,8 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Fístulas intestinais - Como conduzir ?</t>
+    <t xml:space="preserve">
+Deiscências intestinais - Como conduzir ?</t>
   </si>
   <si>
     <t xml:space="preserve">Cláudia Joaquim - RJ</t>
@@ -1129,7 +1252,11 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">14:25 - 14:35</t>
+    <t xml:space="preserve">14:25 - 14:35
+(10 min)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INTERVALO </t>
   </si>
   <si>
     <t xml:space="preserve">14:35 - 16:15
@@ -1148,12 +1275,13 @@
       <rPr>
         <b/>
         <sz val="10"/>
-        <color theme="6" tint="-0.499984740745262"/>
+        <color rgb="FF006400"/>
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">* Hospital Barão de Lucena - PE
-Fabio Ohara - SP </t>
+Fabio Ohara - SP 
+</t>
     </r>
     <r>
       <rPr>
@@ -1163,63 +1291,23 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
+* BOGOTA - Colômbia  
+Santiago Machicado 
+* CUSCO - Peru
+Eric Arancibia
+*Hospital Mocelia - México 
+Armando Menocau  </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Encerramento e Feijoada na Piscina </t>
+  </si>
+  <si>
+    <t xml:space="preserve">08:00 - 10:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRURGIAS AO VIVO - SALA A                                                                                                                                                                   
 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="5" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* BOGOTA - Colômbia  
-Santiago Machicado 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="4" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* CUSCO - Peru
-Eric Arancibia</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF500000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Encerramento e Feijoada na Piscina </t>
-  </si>
-  <si>
-    <t xml:space="preserve">08:00 - 10:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRURGIAS AO VIVO                                                                                                                                                                           
-Presidente : Iolanda Matias - PE 
-Debatedores: Gilvan Santos - PE, Mariana Roma - PE, Felipe Rocha - PE, Guilherme zanluchi SP</t>
   </si>
   <si>
     <t xml:space="preserve">10:30  - 11:10
@@ -1246,6 +1334,9 @@
     <t xml:space="preserve">Lesão vesical - limites da ressecção. Existem repercussões a longo prazo? </t>
   </si>
   <si>
+    <t xml:space="preserve">Arthur Farias - PB</t>
+  </si>
+  <si>
     <t xml:space="preserve">11:00 -11:10              
 (10 min)</t>
   </si>
@@ -1253,10 +1344,20 @@
     <t>Discussão</t>
   </si>
   <si>
-    <t xml:space="preserve">11:10 - 11:40             (30 min)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conferências                                                                                                                                             Presidente : Valter Ivo Paiva PE </t>
+    <r>
+      <t xml:space="preserve">Conferências           
+  Presidente:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FFAC0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Diogenes Fontão - PE </t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">11:10 - 11:25 
@@ -1361,11 +1462,14 @@
 (10 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">12:30 - 13:00
-(1 hora e 10 min) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">INTERVALO (SIMPÓSIO) </t>
+    <t xml:space="preserve">SIMPÓSIO ABIACON - LUNCH BOX  (SALA A) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">12:55 - 13:40
+(45 min) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">INTERVALO LIVRE </t>
   </si>
   <si>
     <t xml:space="preserve">13:40 - 14:20
@@ -1416,15 +1520,14 @@
 (15 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">CIRURGIAS AO VIVO                                                                                                                                                                                        Coordenador : Jardel Soares - PE
-Debatedores : Sidraiton Melo - PE, Andreisa Bilhar - CE, Yole Minervino - PB</t>
+    <t xml:space="preserve">CIRURGIAS AO VIVO  - SALA A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="11.000000"/>
       <name val="Calibri"/>
@@ -1494,13 +1597,26 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10.000000"/>
+      <color rgb="FFAC0000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <i/>
       <sz val="10.000000"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10.000000"/>
+      <color rgb="FFAC0000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1589,6 +1705,24 @@
       <patternFill patternType="solid">
         <fgColor indexed="43"/>
         <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="5"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="5"/>
+        <bgColor rgb="FFFDEADA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="5"/>
+        <bgColor indexed="43"/>
       </patternFill>
     </fill>
   </fills>
@@ -1904,7 +2038,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="153">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1975,13 +2109,13 @@
     <xf fontId="7" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf fontId="7" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf fontId="6" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="7" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="7" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="7" fillId="6" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2059,6 +2193,15 @@
     <xf fontId="6" fillId="5" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf fontId="3" fillId="6" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="6" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="6" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf fontId="3" fillId="6" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2134,6 +2277,27 @@
     <xf fontId="6" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf fontId="11" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="11" fillId="5" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="11" fillId="6" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="11" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="6" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf fontId="10" fillId="12" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2146,143 +2310,185 @@
     <xf fontId="3" fillId="13" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf fontId="11" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="6" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="5" borderId="21" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="9" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="22" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="5" borderId="23" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="17" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="8" fillId="5" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="7" fillId="6" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="4" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="8" fillId="7" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="8" fillId="7" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="8" fillId="7" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="7" fillId="16" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="8" fillId="16" borderId="24" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="13" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="8" fillId="13" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="12" fillId="10" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="11" fillId="17" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="13" fillId="18" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="13" fillId="19" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="10" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="10" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="10" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="0" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="8" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="21" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="11" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="11" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="23" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="11" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="24" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="11" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="10" borderId="10" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="10" borderId="11" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="16" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="16" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="13" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="6" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="15" borderId="15" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="15" borderId="19" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="15" borderId="20" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="16" borderId="24" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf fontId="3" fillId="9" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="7" fillId="5" borderId="21" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="10" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="8" fillId="5" borderId="22" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="7" fillId="5" borderId="23" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="7" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="8" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="8" fillId="5" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="7" fillId="6" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="4" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="8" fillId="7" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="8" fillId="7" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="8" fillId="7" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="7" fillId="16" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="8" fillId="16" borderId="24" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="13" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="8" fillId="13" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="5" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="11" fillId="10" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="10" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="0" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="8" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="8" borderId="21" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="11" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="11" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="8" borderId="23" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="11" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="8" borderId="24" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="8" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="11" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="10" borderId="10" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="10" borderId="11" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="16" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="16" borderId="2" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="13" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="6" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="15" borderId="15" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="15" borderId="19" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="15" borderId="20" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="16" borderId="24" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf fontId="6" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf fontId="3" fillId="6" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="6" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf fontId="3" fillId="0" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="18" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="11" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="11" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="11" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="6" fillId="9" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -2314,7 +2520,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>32</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>74458</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1409698" cy="314350"/>
@@ -2346,7 +2552,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>402168</xdr:colOff>
-      <xdr:row>32</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>107950</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="590549" cy="281350"/>
@@ -2378,7 +2584,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>654050</xdr:colOff>
-      <xdr:row>32</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="985232" cy="425450"/>
@@ -2504,7 +2710,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>99</xdr:row>
       <xdr:rowOff>74458</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1409698" cy="314350"/>
@@ -2536,7 +2742,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>402168</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>99</xdr:row>
       <xdr:rowOff>107950</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="590549" cy="281350"/>
@@ -2568,7 +2774,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>654050</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>99</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="985232" cy="425450"/>
@@ -2690,6 +2896,74 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2768569</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>133200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2768930</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>133560</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Tinta 1"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3858120" y="36033450"/>
+          <a:ext cx="18000" cy="18000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2470130</xdr:colOff>
+      <xdr:row>77</xdr:row>
+      <xdr:rowOff>57080</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2470490</xdr:colOff>
+      <xdr:row>77</xdr:row>
+      <xdr:rowOff>57439</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Tinta 2"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3559680" y="35246130"/>
+          <a:ext cx="18000" cy="18000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3198,12 +3472,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultColWidth="10.26953125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="10.1796875" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" style="2" width="15.7265625"/>
-    <col customWidth="1" min="2" max="2" style="1" width="72.54296875"/>
-    <col customWidth="1" min="3" max="3" style="1" width="29.26953125"/>
-    <col min="4" max="16384" style="1" width="10.26953125"/>
+    <col customWidth="1" min="2" max="2" style="1" width="74.1796875"/>
+    <col customWidth="1" min="3" max="3" style="1" width="28.81640625"/>
+    <col min="4" max="16384" style="1" width="10.1796875"/>
   </cols>
   <sheetData>
     <row r="1" ht="39.649999999999999" customHeight="1">
@@ -3279,10 +3553,10 @@
       <c r="A8" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="25" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3293,15 +3567,15 @@
       <c r="B9" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="25" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="10" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="24" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="27"/>
@@ -3376,18 +3650,20 @@
       <c r="D16" s="28"/>
     </row>
     <row r="17" s="28" customFormat="1" ht="28" customHeight="1">
-      <c r="A17" s="38" t="s">
+      <c r="A17" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="38" t="s">
+      <c r="B17" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="11"/>
+      <c r="C17" s="11" t="s">
+        <v>41</v>
+      </c>
       <c r="D17" s="28"/>
     </row>
     <row r="18" s="28" customFormat="1" ht="28" customHeight="1">
       <c r="A18" s="38" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>22</v>
@@ -3397,29 +3673,29 @@
     </row>
     <row r="19" s="28" customFormat="1" ht="28" customHeight="1">
       <c r="A19" s="38" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D19" s="28"/>
     </row>
     <row r="20" s="28" customFormat="1" ht="38.25" customHeight="1">
       <c r="A20" s="40" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B20" s="41" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C20" s="41"/>
       <c r="D20" s="28"/>
     </row>
     <row r="21" s="42" customFormat="1" ht="28" customHeight="1">
       <c r="A21" s="43" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B21" s="44"/>
       <c r="C21" s="45"/>
@@ -3427,18 +3703,18 @@
     </row>
     <row r="22" s="28" customFormat="1" ht="204" customHeight="1">
       <c r="A22" s="46" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B22" s="47" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C22" s="48" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" s="19" customFormat="1" ht="28" customHeight="1">
       <c r="A23" s="49" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B23" s="50" t="s">
         <v>24</v>
@@ -3447,347 +3723,345 @@
     </row>
     <row r="24" s="8" customFormat="1" ht="42" customHeight="1">
       <c r="A24" s="33" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24" s="34" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C24" s="35"/>
       <c r="D24" s="8"/>
     </row>
     <row r="25" s="8" customFormat="1" ht="28" customHeight="1">
       <c r="A25" s="51" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D25" s="8"/>
     </row>
     <row r="26" s="8" customFormat="1" ht="28" customHeight="1">
       <c r="A26" s="51" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D26" s="8"/>
     </row>
     <row r="27" s="32" customFormat="1" ht="28" customHeight="1">
       <c r="A27" s="51" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D27" s="32"/>
     </row>
     <row r="28" s="32" customFormat="1" ht="28" customHeight="1">
       <c r="A28" s="51" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D28" s="32"/>
     </row>
-    <row r="29" s="8" customFormat="1" ht="28" customHeight="1">
-      <c r="A29" s="51" t="s">
-        <v>66</v>
-      </c>
-      <c r="B29" s="52" t="s">
+    <row r="29" s="32" customFormat="1" ht="28" customHeight="1">
+      <c r="A29" s="52" t="s">
         <v>67</v>
       </c>
-      <c r="C29" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D29" s="8"/>
+      <c r="B29" s="53"/>
+      <c r="C29" s="54"/>
+      <c r="D29" s="32"/>
     </row>
     <row r="30" s="8" customFormat="1" ht="28" customHeight="1">
       <c r="A30" s="51" t="s">
         <v>68</v>
       </c>
-      <c r="B30" s="53" t="s">
+      <c r="B30" s="55" t="s">
         <v>69</v>
       </c>
       <c r="C30" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D30" s="8"/>
+    </row>
+    <row r="31" s="8" customFormat="1" ht="28" customHeight="1">
+      <c r="A31" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="D30" s="8"/>
-    </row>
-    <row r="31" s="19" customFormat="1" ht="79.5" customHeight="1">
-      <c r="A31" s="54" t="s">
+      <c r="B31" s="56" t="s">
         <v>71</v>
       </c>
-      <c r="B31" s="55" t="s">
+      <c r="C31" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C31" s="56" t="s">
+      <c r="D31" s="8"/>
+    </row>
+    <row r="32" s="19" customFormat="1" ht="109" customHeight="1">
+      <c r="A32" s="57" t="s">
         <v>73</v>
-      </c>
-      <c r="D31" s="19"/>
-    </row>
-    <row r="32" s="19" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A32" s="57">
-        <v>0.75347222222222221</v>
       </c>
       <c r="B32" s="58" t="s">
         <v>74</v>
       </c>
-      <c r="C32" s="59"/>
+      <c r="C32" s="59" t="s">
+        <v>75</v>
+      </c>
       <c r="D32" s="19"/>
     </row>
-    <row r="33" s="60" customFormat="1" ht="39.649999999999999" customHeight="1">
-      <c r="A33" s="61" t="s">
+    <row r="33" s="19" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A33" s="60">
+        <v>0.75347222222222221</v>
+      </c>
+      <c r="B33" s="61" t="s">
+        <v>76</v>
+      </c>
+      <c r="C33" s="62"/>
+      <c r="D33" s="19"/>
+    </row>
+    <row r="34" s="63" customFormat="1" ht="39.649999999999999" customHeight="1">
+      <c r="A34" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="B33" s="61"/>
-      <c r="C33" s="61"/>
-    </row>
-    <row r="34" s="4" customFormat="1" ht="25" customHeight="1">
-      <c r="A34" s="5" t="s">
+      <c r="B34" s="64"/>
+      <c r="C34" s="64"/>
+    </row>
+    <row r="35" s="4" customFormat="1" ht="25" customHeight="1">
+      <c r="A35" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B35" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C35" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="35" s="19" customFormat="1" ht="35.149999999999999" customHeight="1">
-      <c r="A35" s="62" t="s">
-        <v>75</v>
-      </c>
-      <c r="B35" s="63"/>
-      <c r="C35" s="64"/>
-      <c r="D35" s="19"/>
-    </row>
-    <row r="36" s="16" customFormat="1" ht="42" customHeight="1">
+    <row r="36" s="19" customFormat="1" ht="35.149999999999999" customHeight="1">
       <c r="A36" s="65" t="s">
-        <v>76</v>
-      </c>
-      <c r="B36" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="C36" s="35"/>
-      <c r="D36" s="16"/>
-    </row>
-    <row r="37" s="16" customFormat="1" ht="28" customHeight="1">
-      <c r="A37" s="66" t="s">
+      <c r="B36" s="66"/>
+      <c r="C36" s="67"/>
+      <c r="D36" s="19"/>
+    </row>
+    <row r="37" s="16" customFormat="1" ht="42" customHeight="1">
+      <c r="A37" s="68" t="s">
         <v>78</v>
       </c>
-      <c r="B37" s="66" t="s">
+      <c r="B37" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="35"/>
+      <c r="D37" s="16"/>
+    </row>
+    <row r="38" s="16" customFormat="1" ht="28" customHeight="1">
+      <c r="A38" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="D37" s="16"/>
-    </row>
-    <row r="38" s="16" customFormat="1" ht="28" customHeight="1">
-      <c r="A38" s="67" t="s">
+      <c r="B38" s="69" t="s">
         <v>81</v>
       </c>
-      <c r="B38" s="66" t="s">
+      <c r="C38" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="C38" s="11" t="s">
+      <c r="D38" s="16"/>
+    </row>
+    <row r="39" s="16" customFormat="1" ht="28" customHeight="1">
+      <c r="A39" s="70" t="s">
         <v>83</v>
       </c>
-      <c r="D38" s="16"/>
-    </row>
-    <row r="39" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A39" s="66" t="s">
+      <c r="B39" s="69" t="s">
         <v>84</v>
       </c>
-      <c r="B39" s="68" t="s">
+      <c r="C39" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="C39" s="37" t="s">
+      <c r="D39" s="16"/>
+    </row>
+    <row r="40" s="19" customFormat="1" ht="28" customHeight="1">
+      <c r="A40" s="69" t="s">
         <v>86</v>
       </c>
-      <c r="D39" s="19"/>
-    </row>
-    <row r="40" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A40" s="68" t="s">
+      <c r="B40" s="71" t="s">
         <v>87</v>
       </c>
-      <c r="B40" s="66" t="s">
+      <c r="C40" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="C40" s="37" t="s">
+      <c r="D40" s="19"/>
+    </row>
+    <row r="41" s="19" customFormat="1" ht="28" customHeight="1">
+      <c r="A41" s="71" t="s">
         <v>89</v>
       </c>
-      <c r="D40" s="19"/>
-    </row>
-    <row r="41" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A41" s="68" t="s">
+      <c r="B41" s="69" t="s">
         <v>90</v>
       </c>
-      <c r="B41" s="66" t="s">
+      <c r="C41" s="37" t="s">
         <v>91</v>
       </c>
-      <c r="C41" s="37" t="s">
+      <c r="D41" s="19"/>
+    </row>
+    <row r="42" s="19" customFormat="1" ht="28" customHeight="1">
+      <c r="A42" s="71" t="s">
         <v>92</v>
       </c>
-      <c r="D41" s="19"/>
-    </row>
-    <row r="42" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A42" s="68" t="s">
+      <c r="B42" s="69" t="s">
         <v>93</v>
       </c>
-      <c r="B42" s="69" t="s">
+      <c r="C42" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="D42" s="19"/>
+    </row>
+    <row r="43" s="19" customFormat="1" ht="28" customHeight="1">
+      <c r="A43" s="71" t="s">
+        <v>95</v>
+      </c>
+      <c r="B43" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="C42" s="69"/>
-      <c r="D42" s="19"/>
-    </row>
-    <row r="43" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A43" s="70" t="s">
-        <v>94</v>
-      </c>
-      <c r="B43" s="71" t="s">
+      <c r="C43" s="72"/>
+      <c r="D43" s="19"/>
+    </row>
+    <row r="44" s="19" customFormat="1" ht="28" customHeight="1">
+      <c r="A44" s="73" t="s">
+        <v>96</v>
+      </c>
+      <c r="B44" s="74" t="s">
         <v>24</v>
       </c>
-      <c r="C43" s="71"/>
-      <c r="D43" s="19"/>
-    </row>
-    <row r="44" s="72" customFormat="1" ht="28" customHeight="1">
-      <c r="A44" s="70" t="s">
-        <v>95</v>
-      </c>
-      <c r="B44" s="73" t="s">
-        <v>96</v>
-      </c>
       <c r="C44" s="74"/>
-      <c r="D44" s="72"/>
-    </row>
-    <row r="45" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A45" s="75" t="s">
+      <c r="D44" s="19"/>
+    </row>
+    <row r="45" s="75" customFormat="1" ht="28" customHeight="1">
+      <c r="A45" s="73" t="s">
         <v>97</v>
       </c>
-      <c r="B45" s="66" t="s">
+      <c r="B45" s="76" t="s">
         <v>98</v>
       </c>
-      <c r="C45" s="76" t="s">
+      <c r="C45" s="77"/>
+      <c r="D45" s="75"/>
+    </row>
+    <row r="46" s="19" customFormat="1" ht="28" customHeight="1">
+      <c r="A46" s="78" t="s">
         <v>99</v>
       </c>
-      <c r="D45" s="19"/>
-    </row>
-    <row r="46" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A46" s="75" t="s">
+      <c r="B46" s="69" t="s">
         <v>100</v>
       </c>
-      <c r="B46" s="66" t="s">
+      <c r="C46" s="79" t="s">
         <v>101</v>
       </c>
-      <c r="C46" s="76" t="s">
+      <c r="D46" s="19"/>
+    </row>
+    <row r="47" s="19" customFormat="1" ht="28" customHeight="1">
+      <c r="A47" s="78" t="s">
         <v>102</v>
       </c>
-      <c r="D46" s="19"/>
-    </row>
-    <row r="47" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A47" s="75" t="s">
+      <c r="B47" s="69" t="s">
         <v>103</v>
       </c>
-      <c r="B47" s="66" t="s">
+      <c r="C47" s="79" t="s">
         <v>104</v>
       </c>
-      <c r="C47" s="76"/>
       <c r="D47" s="19"/>
     </row>
-    <row r="48" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A48" s="75" t="s">
+    <row r="48" s="80" customFormat="1" ht="28" customHeight="1">
+      <c r="A48" s="81" t="s">
         <v>105</v>
       </c>
-      <c r="B48" s="66" t="s">
+      <c r="B48" s="82" t="s">
         <v>106</v>
       </c>
-      <c r="C48" s="76" t="s">
+      <c r="C48" s="83" t="s">
         <v>107</v>
       </c>
-      <c r="D48" s="19"/>
+      <c r="D48" s="80"/>
     </row>
     <row r="49" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A49" s="75" t="s">
+      <c r="A49" s="78" t="s">
         <v>108</v>
       </c>
-      <c r="B49" s="66" t="s">
+      <c r="B49" s="69" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="76" t="s">
+      <c r="C49" s="79" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="19"/>
     </row>
     <row r="50" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A50" s="75" t="s">
+      <c r="A50" s="78" t="s">
         <v>111</v>
       </c>
-      <c r="B50" s="66" t="s">
+      <c r="B50" s="69" t="s">
         <v>112</v>
       </c>
-      <c r="C50" s="76" t="s">
+      <c r="C50" s="79" t="s">
         <v>113</v>
       </c>
       <c r="D50" s="19"/>
     </row>
     <row r="51" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A51" s="75" t="s">
+      <c r="A51" s="78" t="s">
         <v>114</v>
       </c>
-      <c r="B51" s="66" t="s">
+      <c r="B51" s="69" t="s">
         <v>115</v>
       </c>
-      <c r="C51" s="76" t="s">
-        <v>44</v>
+      <c r="C51" s="79" t="s">
+        <v>116</v>
       </c>
       <c r="D51" s="19"/>
     </row>
-    <row r="52" s="19" customFormat="1" ht="37.5" customHeight="1">
-      <c r="A52" s="70" t="s">
-        <v>116</v>
-      </c>
-      <c r="B52" s="50" t="s">
-        <v>46</v>
-      </c>
-      <c r="C52" s="50"/>
-      <c r="D52" s="19"/>
+    <row r="52" s="84" customFormat="1" ht="28" customHeight="1">
+      <c r="A52" s="85" t="s">
+        <v>117</v>
+      </c>
+      <c r="B52" s="86" t="s">
+        <v>47</v>
+      </c>
+      <c r="C52" s="86"/>
+      <c r="D52" s="84"/>
     </row>
     <row r="53" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A53" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="B53" s="77"/>
-      <c r="C53" s="77"/>
+      <c r="A53" s="87" t="s">
+        <v>48</v>
+      </c>
+      <c r="B53" s="87"/>
+      <c r="C53" s="87"/>
       <c r="D53" s="19"/>
     </row>
-    <row r="54" s="19" customFormat="1" ht="55.5" customHeight="1">
-      <c r="A54" s="78" t="s">
-        <v>48</v>
-      </c>
-      <c r="B54" s="79" t="s">
-        <v>117</v>
-      </c>
-      <c r="C54" s="80"/>
+    <row r="54" s="19" customFormat="1" ht="29.149999999999999" customHeight="1">
+      <c r="A54" s="88" t="s">
+        <v>49</v>
+      </c>
+      <c r="B54" s="89" t="s">
+        <v>118</v>
+      </c>
+      <c r="C54" s="90"/>
       <c r="D54" s="19"/>
     </row>
     <row r="55" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A55" s="70" t="s">
-        <v>51</v>
+      <c r="A55" s="73" t="s">
+        <v>52</v>
       </c>
       <c r="B55" s="50" t="s">
         <v>24</v>
@@ -3795,709 +4069,737 @@
       <c r="C55" s="50"/>
       <c r="D55" s="19"/>
     </row>
-    <row r="56" s="16" customFormat="1" ht="42" customHeight="1">
-      <c r="A56" s="65" t="s">
-        <v>118</v>
-      </c>
-      <c r="B56" s="81" t="s">
+    <row r="56" s="80" customFormat="1" ht="28" customHeight="1">
+      <c r="A56" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="C56" s="81"/>
-      <c r="D56" s="16"/>
-    </row>
-    <row r="57" s="19" customFormat="1" ht="20.25" customHeight="1">
-      <c r="A57" s="82" t="s">
+      <c r="B56" s="79" t="s">
         <v>120</v>
       </c>
-      <c r="B57" s="83" t="s">
+      <c r="C56" s="79" t="s">
+        <v>45</v>
+      </c>
+      <c r="D56" s="80"/>
+    </row>
+    <row r="57" s="91" customFormat="1" ht="42" customHeight="1">
+      <c r="A57" s="92" t="s">
         <v>121</v>
       </c>
-      <c r="C57" s="84"/>
-      <c r="D57" s="19"/>
-    </row>
-    <row r="58" s="19" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A58" s="85"/>
-      <c r="B58" s="86" t="s">
+      <c r="B57" s="93" t="s">
         <v>122</v>
       </c>
-      <c r="C58" s="76" t="s">
+      <c r="C57" s="93"/>
+      <c r="D57" s="91"/>
+    </row>
+    <row r="58" s="80" customFormat="1" ht="20.25" customHeight="1">
+      <c r="A58" s="94" t="s">
         <v>123</v>
       </c>
-      <c r="D58" s="19"/>
-    </row>
-    <row r="59" s="28" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A59" s="85"/>
-      <c r="B59" s="86" t="s">
+      <c r="B58" s="95" t="s">
         <v>124</v>
       </c>
-      <c r="C59" s="76" t="s">
+      <c r="C58" s="96"/>
+      <c r="D58" s="80"/>
+    </row>
+    <row r="59" s="80" customFormat="1" ht="27.75" customHeight="1">
+      <c r="A59" s="97"/>
+      <c r="B59" s="79" t="s">
         <v>125</v>
       </c>
-      <c r="D59" s="28"/>
-    </row>
-    <row r="60" s="19" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A60" s="75" t="s">
+      <c r="C59" s="79" t="s">
         <v>126</v>
       </c>
-      <c r="B60" s="86" t="s">
+      <c r="D59" s="80"/>
+    </row>
+    <row r="60" s="80" customFormat="1" ht="27.75" customHeight="1">
+      <c r="A60" s="97"/>
+      <c r="B60" s="79" t="s">
         <v>127</v>
       </c>
-      <c r="C60" s="76" t="s">
+      <c r="C60" s="98"/>
+      <c r="D60" s="80"/>
+    </row>
+    <row r="61" s="80" customFormat="1" ht="27.75" customHeight="1">
+      <c r="A61" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="D60" s="19"/>
-    </row>
-    <row r="61" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A61" s="75" t="s">
+      <c r="B61" s="79" t="s">
         <v>129</v>
       </c>
-      <c r="B61" s="66" t="s">
+      <c r="C61" s="79" t="s">
         <v>130</v>
       </c>
-      <c r="C61" s="76" t="s">
+      <c r="D61" s="80"/>
+    </row>
+    <row r="62" s="80" customFormat="1" ht="28" customHeight="1">
+      <c r="A62" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="D61" s="19"/>
-    </row>
-    <row r="62" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A62" s="75" t="s">
+      <c r="B62" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="B62" s="86" t="s">
+      <c r="C62" s="79" t="s">
+        <v>133</v>
+      </c>
+      <c r="D62" s="80"/>
+    </row>
+    <row r="63" s="80" customFormat="1" ht="28" customHeight="1">
+      <c r="A63" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B63" s="79" t="s">
         <v>22</v>
       </c>
-      <c r="C62" s="87"/>
-      <c r="D62" s="19"/>
-    </row>
-    <row r="63" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A63" s="75" t="s">
-        <v>133</v>
-      </c>
-      <c r="B63" s="86" t="s">
+      <c r="C63" s="99"/>
+      <c r="D63" s="80"/>
+    </row>
+    <row r="64" s="80" customFormat="1" ht="28" customHeight="1">
+      <c r="A64" s="51" t="s">
         <v>134</v>
       </c>
-      <c r="C63" s="76" t="s">
-        <v>44</v>
-      </c>
-      <c r="D63" s="19"/>
-    </row>
-    <row r="64" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A64" s="67" t="s">
+      <c r="B64" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="B64" s="66" t="s">
+      <c r="C64" s="79" t="s">
+        <v>94</v>
+      </c>
+      <c r="D64" s="80"/>
+    </row>
+    <row r="65" s="80" customFormat="1" ht="28" customHeight="1">
+      <c r="A65" s="51"/>
+      <c r="B65" s="100" t="s">
         <v>136</v>
       </c>
-      <c r="C64" s="86"/>
-      <c r="D64" s="19"/>
-    </row>
-    <row r="65" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A65" s="67"/>
-      <c r="B65" s="88" t="s">
+      <c r="C65" s="79" t="s">
+        <v>45</v>
+      </c>
+      <c r="D65" s="80"/>
+    </row>
+    <row r="66" s="80" customFormat="1" ht="28" customHeight="1">
+      <c r="A66" s="51"/>
+      <c r="B66" s="100" t="s">
         <v>137</v>
       </c>
-      <c r="C65" s="86"/>
-      <c r="D65" s="19"/>
-    </row>
-    <row r="66" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A66" s="67"/>
-      <c r="B66" s="88" t="s">
+      <c r="C66" s="79" t="s">
         <v>138</v>
       </c>
-      <c r="C66" s="76" t="s">
+      <c r="D66" s="80"/>
+    </row>
+    <row r="67" s="80" customFormat="1" ht="28" customHeight="1">
+      <c r="A67" s="51"/>
+      <c r="B67" s="100" t="s">
         <v>139</v>
       </c>
-      <c r="D66" s="19"/>
-    </row>
-    <row r="67" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A67" s="67"/>
-      <c r="B67" s="88" t="s">
+      <c r="C67" s="79" t="s">
         <v>140</v>
       </c>
-      <c r="C67" s="76" t="s">
+      <c r="D67" s="80"/>
+    </row>
+    <row r="68" s="80" customFormat="1" ht="28" customHeight="1">
+      <c r="A68" s="51">
+        <v>0.75694444444444453</v>
+      </c>
+      <c r="B68" s="100" t="s">
         <v>141</v>
       </c>
-      <c r="D67" s="19"/>
-    </row>
-    <row r="68" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A68" s="67">
-        <v>0.75</v>
-      </c>
-      <c r="B68" s="88" t="s">
-        <v>142</v>
-      </c>
-      <c r="C68" s="86"/>
-      <c r="D68" s="19"/>
+      <c r="C68" s="79"/>
+      <c r="D68" s="80"/>
     </row>
     <row r="69" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A69" s="89" t="s">
-        <v>74</v>
-      </c>
-      <c r="B69" s="89"/>
-      <c r="C69" s="89"/>
+      <c r="A69" s="101" t="s">
+        <v>76</v>
+      </c>
+      <c r="B69" s="101"/>
+      <c r="C69" s="101"/>
       <c r="D69" s="19"/>
     </row>
     <row r="70" s="19" customFormat="1" ht="28" customHeight="1">
-      <c r="A70" s="90"/>
-      <c r="B70" s="90"/>
-      <c r="C70" s="90"/>
+      <c r="A70" s="102"/>
+      <c r="B70" s="102"/>
+      <c r="C70" s="102"/>
       <c r="D70" s="19"/>
     </row>
-    <row r="71" s="60" customFormat="1" ht="39.649999999999999" customHeight="1">
-      <c r="A71" s="61" t="s">
+    <row r="71" s="63" customFormat="1" ht="39.649999999999999" customHeight="1">
+      <c r="A71" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="B71" s="61"/>
-      <c r="C71" s="61"/>
-    </row>
-    <row r="72" s="91" customFormat="1" ht="28" customHeight="1">
+      <c r="B71" s="64"/>
+      <c r="C71" s="64"/>
+    </row>
+    <row r="72" s="103" customFormat="1" ht="28" customHeight="1">
       <c r="A72" s="5" t="s">
         <v>1</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C72" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D72" s="91"/>
-    </row>
-    <row r="73" s="60" customFormat="1" ht="35.149999999999999" customHeight="1">
-      <c r="A73" s="92" t="s">
+      <c r="D72" s="103"/>
+    </row>
+    <row r="73" s="63" customFormat="1" ht="35.149999999999999" customHeight="1">
+      <c r="A73" s="104" t="s">
         <v>9</v>
       </c>
-      <c r="B73" s="93"/>
-      <c r="C73" s="94"/>
-    </row>
-    <row r="74" s="95" customFormat="1" ht="221" customHeight="1">
-      <c r="A74" s="96" t="s">
+      <c r="B73" s="105"/>
+      <c r="C73" s="106"/>
+    </row>
+    <row r="74" s="107" customFormat="1" ht="205.5" customHeight="1">
+      <c r="A74" s="108" t="s">
+        <v>143</v>
+      </c>
+      <c r="B74" s="109" t="s">
         <v>144</v>
       </c>
-      <c r="B74" s="97" t="s">
+      <c r="C74" s="110" t="s">
         <v>145</v>
       </c>
-      <c r="C74" s="98" t="s">
+      <c r="D74" s="107"/>
+    </row>
+    <row r="75" s="42" customFormat="1" ht="28" customHeight="1">
+      <c r="A75" s="85" t="s">
         <v>146</v>
       </c>
-      <c r="D74" s="95"/>
-    </row>
-    <row r="75" s="42" customFormat="1" ht="28" customHeight="1">
-      <c r="A75" s="99" t="s">
+      <c r="B75" s="99" t="s">
+        <v>24</v>
+      </c>
+      <c r="C75" s="99"/>
+      <c r="D75" s="42"/>
+    </row>
+    <row r="76" s="42" customFormat="1" ht="32.149999999999999" customHeight="1">
+      <c r="A76" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="B75" s="87" t="s">
-        <v>24</v>
-      </c>
-      <c r="C75" s="87"/>
-      <c r="D75" s="42"/>
-    </row>
-    <row r="76" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A76" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="B76" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="C76" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="D76" s="12"/>
+      <c r="B76" s="112"/>
+      <c r="C76" s="113"/>
+      <c r="D76" s="42"/>
     </row>
     <row r="77" s="12" customFormat="1" ht="28" customHeight="1">
       <c r="A77" s="9" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B77" s="38" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C77" s="11" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D77" s="12"/>
     </row>
     <row r="78" s="12" customFormat="1" ht="28" customHeight="1">
       <c r="A78" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="B78" s="38" t="s">
+        <v>152</v>
+      </c>
+      <c r="C78" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D78" s="12"/>
+    </row>
+    <row r="79" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A79" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="B78" s="38" t="s">
+      <c r="B79" s="38" t="s">
         <v>155</v>
       </c>
-      <c r="C78" s="11" t="s">
+      <c r="C79" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="D78" s="12"/>
-    </row>
-    <row r="79" s="8" customFormat="1" ht="42" customHeight="1">
-      <c r="A79" s="33" t="s">
+      <c r="D79" s="12"/>
+    </row>
+    <row r="80" s="8" customFormat="1" ht="42" customHeight="1">
+      <c r="A80" s="33" t="s">
         <v>157</v>
       </c>
-      <c r="B79" s="34" t="s">
+      <c r="B80" s="34" t="s">
         <v>158</v>
       </c>
-      <c r="C79" s="35"/>
-      <c r="D79" s="8"/>
-    </row>
-    <row r="80" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A80" s="51" t="s">
-        <v>159</v>
-      </c>
-      <c r="B80" s="38" t="s">
-        <v>160</v>
-      </c>
-      <c r="C80" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="D80" s="12"/>
+      <c r="C80" s="35"/>
+      <c r="D80" s="8"/>
     </row>
     <row r="81" s="12" customFormat="1" ht="28" customHeight="1">
       <c r="A81" s="51" t="s">
+        <v>159</v>
+      </c>
+      <c r="B81" s="38" t="s">
+        <v>160</v>
+      </c>
+      <c r="C81" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="D81" s="12"/>
+    </row>
+    <row r="82" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A82" s="51" t="s">
         <v>162</v>
       </c>
-      <c r="B81" s="38" t="s">
+      <c r="B82" s="38" t="s">
         <v>163</v>
       </c>
-      <c r="C81" s="11" t="s">
+      <c r="C82" s="11" t="s">
         <v>164</v>
-      </c>
-      <c r="D81" s="12"/>
-    </row>
-    <row r="82" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A82" s="37" t="s">
-        <v>165</v>
-      </c>
-      <c r="B82" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="C82" s="37" t="s">
-        <v>113</v>
       </c>
       <c r="D82" s="12"/>
     </row>
     <row r="83" s="12" customFormat="1" ht="28" customHeight="1">
       <c r="A83" s="37" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B83" s="38" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C83" s="37" t="s">
-        <v>169</v>
+        <v>116</v>
       </c>
       <c r="D83" s="12"/>
     </row>
     <row r="84" s="12" customFormat="1" ht="28" customHeight="1">
       <c r="A84" s="37" t="s">
+        <v>167</v>
+      </c>
+      <c r="B84" s="38" t="s">
+        <v>168</v>
+      </c>
+      <c r="C84" s="37" t="s">
+        <v>169</v>
+      </c>
+      <c r="D84" s="12"/>
+    </row>
+    <row r="85" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A85" s="37" t="s">
         <v>170</v>
       </c>
-      <c r="B84" s="100" t="s">
+      <c r="B85" s="114" t="s">
         <v>22</v>
       </c>
-      <c r="C84" s="37"/>
-      <c r="D84" s="12"/>
-    </row>
-    <row r="85" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A85" s="101" t="s">
+      <c r="C85" s="37"/>
+      <c r="D85" s="12"/>
+    </row>
+    <row r="86" s="115" customFormat="1" ht="28" customHeight="1">
+      <c r="A86" s="116" t="s">
         <v>171</v>
       </c>
-      <c r="B85" s="41" t="s">
+      <c r="B86" s="117" t="s">
         <v>172</v>
       </c>
-      <c r="C85" s="41"/>
-      <c r="D85" s="12"/>
-    </row>
-    <row r="86" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A86" s="102" t="s">
+      <c r="C86" s="117"/>
+      <c r="D86" s="115"/>
+    </row>
+    <row r="87" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A87" s="118" t="s">
         <v>173</v>
       </c>
-      <c r="B86" s="38" t="s">
+      <c r="B87" s="119"/>
+      <c r="C87" s="120"/>
+      <c r="D87" s="12"/>
+    </row>
+    <row r="88" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A88" s="121" t="s">
         <v>174</v>
       </c>
-      <c r="C86" s="11" t="s">
+      <c r="B88" s="38" t="s">
         <v>175</v>
       </c>
-      <c r="D86" s="12"/>
-    </row>
-    <row r="87" s="12" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A87" s="102" t="s">
+      <c r="C88" s="11" t="s">
         <v>176</v>
       </c>
-      <c r="B87" s="103" t="s">
+      <c r="D88" s="12"/>
+    </row>
+    <row r="89" s="12" customFormat="1" ht="27.75" customHeight="1">
+      <c r="A89" s="121" t="s">
         <v>177</v>
       </c>
-      <c r="C87" s="11" t="s">
+      <c r="B89" s="122" t="s">
         <v>178</v>
       </c>
-      <c r="D87" s="12"/>
-    </row>
-    <row r="88" s="8" customFormat="1" ht="42" customHeight="1">
-      <c r="A88" s="104" t="s">
+      <c r="C89" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="B88" s="34" t="s">
+      <c r="D89" s="12"/>
+    </row>
+    <row r="90" s="8" customFormat="1" ht="42" customHeight="1">
+      <c r="A90" s="123" t="s">
         <v>180</v>
       </c>
-      <c r="C88" s="35"/>
-      <c r="D88" s="8"/>
-    </row>
-    <row r="89" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A89" s="105" t="s">
+      <c r="B90" s="34" t="s">
         <v>181</v>
       </c>
-      <c r="B89" s="106" t="s">
+      <c r="C90" s="35"/>
+      <c r="D90" s="8"/>
+    </row>
+    <row r="91" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A91" s="124" t="s">
         <v>182</v>
       </c>
-      <c r="C89" s="107"/>
-    </row>
-    <row r="90" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A90" s="108"/>
-      <c r="B90" s="109" t="s">
+      <c r="B91" s="125" t="s">
         <v>183</v>
       </c>
-      <c r="C90" s="109" t="s">
+      <c r="C91" s="126"/>
+    </row>
+    <row r="92" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A92" s="127"/>
+      <c r="B92" s="128" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="91" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A91" s="108"/>
-      <c r="B91" s="109" t="s">
+      <c r="C92" s="128" t="s">
         <v>185</v>
       </c>
-      <c r="C91" s="109" t="s">
+    </row>
+    <row r="93" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A93" s="127"/>
+      <c r="B93" s="128" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="92" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A92" s="110"/>
-      <c r="B92" s="109" t="s">
+      <c r="C93" s="128" t="s">
         <v>187</v>
       </c>
-      <c r="C92" s="109" t="s">
+    </row>
+    <row r="94" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A94" s="129"/>
+      <c r="B94" s="128" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="93" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A93" s="111" t="s">
+      <c r="C94" s="128" t="s">
         <v>189</v>
       </c>
-      <c r="B93" s="109" t="s">
+    </row>
+    <row r="95" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A95" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="C93" s="109" t="s">
+      <c r="B95" s="128" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="94" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A94" s="111" t="s">
+      <c r="C95" s="128" t="s">
         <v>192</v>
       </c>
-      <c r="B94" s="112" t="s">
+    </row>
+    <row r="96" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A96" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="B96" s="130" t="s">
         <v>22</v>
       </c>
-      <c r="C94" s="41"/>
-    </row>
-    <row r="95" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A95" s="40" t="s">
-        <v>193</v>
-      </c>
-      <c r="B95" s="113" t="s">
-        <v>172</v>
-      </c>
-      <c r="C95" s="114"/>
-      <c r="D95" s="12"/>
-    </row>
-    <row r="96" s="115" customFormat="1" ht="149.25" customHeight="1">
-      <c r="A96" s="116" t="s">
+      <c r="C96" s="41"/>
+    </row>
+    <row r="97" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A97" s="40" t="s">
         <v>194</v>
       </c>
-      <c r="B96" s="97" t="s">
+      <c r="B97" s="131" t="s">
         <v>195</v>
       </c>
-      <c r="C96" s="117" t="s">
+      <c r="C97" s="132"/>
+      <c r="D97" s="12"/>
+    </row>
+    <row r="98" s="133" customFormat="1" ht="198" customHeight="1">
+      <c r="A98" s="134" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="97" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A97" s="51">
+      <c r="B98" s="109" t="s">
+        <v>197</v>
+      </c>
+      <c r="C98" s="135" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="99" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A99" s="51">
         <v>0.67708333333333337</v>
       </c>
-      <c r="B97" s="118" t="s">
-        <v>197</v>
-      </c>
-      <c r="C97" s="118"/>
-      <c r="D97" s="12"/>
-    </row>
-    <row r="98" s="12" customFormat="1" ht="39.649999999999999" customHeight="1">
-      <c r="A98" s="3" t="s">
+      <c r="B99" s="136" t="s">
+        <v>199</v>
+      </c>
+      <c r="C99" s="136"/>
+      <c r="D99" s="12"/>
+    </row>
+    <row r="100" s="12" customFormat="1" ht="39.649999999999999" customHeight="1">
+      <c r="A100" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B98" s="3"/>
-      <c r="C98" s="3"/>
-    </row>
-    <row r="99" s="91" customFormat="1" ht="28" customHeight="1">
-      <c r="A99" s="5" t="s">
+      <c r="B100" s="3"/>
+      <c r="C100" s="3"/>
+    </row>
+    <row r="101" s="103" customFormat="1" ht="28" customHeight="1">
+      <c r="A101" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B99" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="C99" s="7" t="s">
+      <c r="B101" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="C101" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D99" s="91"/>
-    </row>
-    <row r="100" s="42" customFormat="1" ht="35.149999999999999" customHeight="1">
-      <c r="A100" s="119" t="s">
-        <v>75</v>
-      </c>
-      <c r="B100" s="120"/>
-      <c r="C100" s="121"/>
-      <c r="D100" s="42"/>
-    </row>
-    <row r="101" s="115" customFormat="1" ht="60.75" customHeight="1">
-      <c r="A101" s="122" t="s">
-        <v>198</v>
-      </c>
-      <c r="B101" s="79" t="s">
-        <v>199</v>
-      </c>
-      <c r="C101" s="80"/>
-      <c r="D101" s="115"/>
-    </row>
-    <row r="102" s="42" customFormat="1" ht="28" customHeight="1">
-      <c r="A102" s="99" t="s">
-        <v>147</v>
-      </c>
-      <c r="B102" s="87" t="s">
+      <c r="D101" s="103"/>
+    </row>
+    <row r="102" s="42" customFormat="1" ht="35.149999999999999" customHeight="1">
+      <c r="A102" s="137" t="s">
+        <v>77</v>
+      </c>
+      <c r="B102" s="138"/>
+      <c r="C102" s="139"/>
+      <c r="D102" s="42"/>
+    </row>
+    <row r="103" s="133" customFormat="1" ht="26.149999999999999" customHeight="1">
+      <c r="A103" s="140" t="s">
+        <v>200</v>
+      </c>
+      <c r="B103" s="89" t="s">
+        <v>201</v>
+      </c>
+      <c r="C103" s="90"/>
+      <c r="D103" s="133"/>
+    </row>
+    <row r="104" s="42" customFormat="1" ht="28" customHeight="1">
+      <c r="A104" s="85" t="s">
+        <v>146</v>
+      </c>
+      <c r="B104" s="99" t="s">
         <v>24</v>
       </c>
-      <c r="C102" s="87"/>
-      <c r="D102" s="42"/>
-    </row>
-    <row r="103" s="12" customFormat="1" ht="42" customHeight="1">
-      <c r="A103" s="33" t="s">
-        <v>200</v>
-      </c>
-      <c r="B103" s="81" t="s">
-        <v>201</v>
-      </c>
-      <c r="C103" s="81"/>
-      <c r="D103" s="12"/>
-    </row>
-    <row r="104" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A104" s="102" t="s">
+      <c r="C104" s="99"/>
+      <c r="D104" s="42"/>
+    </row>
+    <row r="105" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A105" s="33" t="s">
         <v>202</v>
       </c>
-      <c r="B104" s="38" t="s">
+      <c r="B105" s="141" t="s">
         <v>203</v>
       </c>
-      <c r="C104" s="11" t="s">
+      <c r="C105" s="141"/>
+      <c r="D105" s="12"/>
+    </row>
+    <row r="106" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A106" s="121" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="105" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A105" s="102" t="s">
+      <c r="B106" s="38" t="s">
+        <v>205</v>
+      </c>
+      <c r="C106" s="11" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="107" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A107" s="121" t="s">
         <v>33</v>
       </c>
-      <c r="B105" s="123" t="s">
-        <v>205</v>
-      </c>
-      <c r="C105" s="11"/>
-    </row>
-    <row r="106" s="42" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A106" s="51" t="s">
-        <v>206</v>
-      </c>
-      <c r="B106" s="118" t="s">
+      <c r="B107" s="142" t="s">
         <v>207</v>
       </c>
-      <c r="C106" s="124"/>
-    </row>
-    <row r="107" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A107" s="9" t="s">
+      <c r="C107" s="82" t="s">
         <v>208</v>
       </c>
-      <c r="B107" s="125" t="s">
+    </row>
+    <row r="108" s="42" customFormat="1" ht="27.75" customHeight="1">
+      <c r="A108" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="C107" s="126"/>
-      <c r="D107" s="12"/>
-    </row>
-    <row r="108" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A108" s="9" t="s">
+      <c r="B108" s="136" t="s">
         <v>210</v>
       </c>
-      <c r="B108" s="38" t="s">
+      <c r="C108" s="143"/>
+    </row>
+    <row r="109" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A109" s="144" t="s">
         <v>211</v>
       </c>
-      <c r="C108" s="11" t="s">
+      <c r="B109" s="145"/>
+      <c r="C109" s="146"/>
+      <c r="D109" s="12"/>
+    </row>
+    <row r="110" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A110" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="D108" s="12"/>
-    </row>
-    <row r="109" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A109" s="9" t="s">
+      <c r="B110" s="38" t="s">
         <v>213</v>
       </c>
-      <c r="B109" s="38" t="s">
+      <c r="C110" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="C109" s="11" t="s">
+      <c r="D110" s="12"/>
+    </row>
+    <row r="111" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A111" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="D109" s="12"/>
-    </row>
-    <row r="110" s="12" customFormat="1" ht="42" customHeight="1">
-      <c r="A110" s="33" t="s">
+      <c r="B111" s="38" t="s">
         <v>216</v>
       </c>
-      <c r="B110" s="34" t="s">
+      <c r="C111" s="11" t="s">
         <v>217</v>
       </c>
-      <c r="C110" s="35"/>
-    </row>
-    <row r="111" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A111" s="51" t="s">
+      <c r="D111" s="12"/>
+    </row>
+    <row r="112" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A112" s="33" t="s">
         <v>218</v>
       </c>
-      <c r="B111" s="123" t="s">
+      <c r="B112" s="34" t="s">
         <v>219</v>
       </c>
-      <c r="C111" s="11" t="s">
+      <c r="C112" s="35"/>
+    </row>
+    <row r="113" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A113" s="51" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="112" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A112" s="51" t="s">
+      <c r="B113" s="142" t="s">
         <v>221</v>
       </c>
-      <c r="B112" s="123" t="s">
+      <c r="C113" s="11" t="s">
         <v>222</v>
       </c>
-      <c r="C112" s="11" t="s">
+    </row>
+    <row r="114" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A114" s="51" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="113" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A113" s="37" t="s">
+      <c r="B114" s="142" t="s">
         <v>224</v>
       </c>
-      <c r="B113" s="123" t="s">
+      <c r="C114" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="C113" s="37" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="114" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A114" s="37" t="s">
-        <v>227</v>
-      </c>
-      <c r="B114" s="38" t="s">
-        <v>228</v>
-      </c>
-      <c r="C114" s="37"/>
     </row>
     <row r="115" s="12" customFormat="1" ht="28" customHeight="1">
       <c r="A115" s="37" t="s">
+        <v>226</v>
+      </c>
+      <c r="B115" s="142" t="s">
+        <v>227</v>
+      </c>
+      <c r="C115" s="37" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="116" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A116" s="37" t="s">
         <v>229</v>
       </c>
-      <c r="B115" s="123" t="s">
+      <c r="B116" s="38" t="s">
+        <v>230</v>
+      </c>
+      <c r="C116" s="147"/>
+    </row>
+    <row r="117" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A117" s="37" t="s">
+        <v>231</v>
+      </c>
+      <c r="B117" s="142" t="s">
         <v>22</v>
       </c>
-      <c r="C115" s="37"/>
-    </row>
-    <row r="116" s="12" customFormat="1" ht="42.75" customHeight="1">
-      <c r="A116" s="40" t="s">
-        <v>230</v>
-      </c>
-      <c r="B116" s="41" t="s">
-        <v>231</v>
-      </c>
-      <c r="C116" s="41"/>
-      <c r="D116" s="12"/>
-    </row>
-    <row r="117" s="12" customFormat="1" ht="42" customHeight="1">
-      <c r="A117" s="33" t="s">
+      <c r="C117" s="37"/>
+    </row>
+    <row r="118" s="12" customFormat="1" ht="25.5" customHeight="1">
+      <c r="A118" s="40" t="s">
+        <v>171</v>
+      </c>
+      <c r="B118" s="148" t="s">
         <v>232</v>
       </c>
-      <c r="B117" s="34" t="s">
+      <c r="C118" s="148"/>
+      <c r="D118" s="12"/>
+    </row>
+    <row r="119" s="12" customFormat="1" ht="28.5" customHeight="1">
+      <c r="A119" s="40" t="s">
         <v>233</v>
       </c>
-      <c r="C117" s="127"/>
-    </row>
-    <row r="118" s="42" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A118" s="102" t="s">
+      <c r="B119" s="149" t="s">
         <v>234</v>
       </c>
-      <c r="B118" s="118" t="s">
+      <c r="C119" s="150"/>
+      <c r="D119" s="12"/>
+    </row>
+    <row r="120" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A120" s="33" t="s">
         <v>235</v>
       </c>
-      <c r="C118" s="128" t="s">
+      <c r="B120" s="34" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="119" s="42" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A119" s="102" t="s">
+      <c r="C120" s="151"/>
+    </row>
+    <row r="121" s="42" customFormat="1" ht="27.75" customHeight="1">
+      <c r="A121" s="121" t="s">
         <v>237</v>
       </c>
-      <c r="B119" s="118" t="s">
+      <c r="B121" s="136" t="s">
         <v>238</v>
       </c>
-      <c r="C119" s="128" t="s">
+      <c r="C121" s="152" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="120" s="42" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A120" s="36" t="s">
+    <row r="122" s="42" customFormat="1" ht="27.75" customHeight="1">
+      <c r="A122" s="121" t="s">
         <v>240</v>
       </c>
-      <c r="B120" s="118" t="s">
+      <c r="B122" s="136" t="s">
         <v>241</v>
       </c>
-      <c r="C120" s="128" t="s">
+      <c r="C122" s="152" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="121" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A121" s="36" t="s">
+    <row r="123" s="42" customFormat="1" ht="27.75" customHeight="1">
+      <c r="A123" s="36" t="s">
         <v>243</v>
       </c>
-      <c r="B121" s="123" t="s">
+      <c r="B123" s="136" t="s">
+        <v>244</v>
+      </c>
+      <c r="C123" s="152" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="124" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A124" s="36" t="s">
+        <v>246</v>
+      </c>
+      <c r="B124" s="142" t="s">
         <v>22</v>
       </c>
-      <c r="C121" s="11"/>
-    </row>
-    <row r="122" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A122" s="40" t="s">
-        <v>244</v>
-      </c>
-      <c r="B122" s="113" t="s">
-        <v>172</v>
-      </c>
-      <c r="C122" s="114"/>
-      <c r="D122" s="12"/>
-    </row>
-    <row r="123" s="115" customFormat="1" ht="58.5" customHeight="1">
-      <c r="A123" s="116" t="s">
-        <v>194</v>
-      </c>
-      <c r="B123" s="79" t="s">
-        <v>245</v>
-      </c>
-      <c r="C123" s="80"/>
-    </row>
-    <row r="124" s="12" customFormat="1" ht="28" customHeight="1">
-      <c r="A124" s="51">
+      <c r="C124" s="11"/>
+    </row>
+    <row r="125" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A125" s="40" t="s">
+        <v>247</v>
+      </c>
+      <c r="B125" s="131" t="s">
+        <v>195</v>
+      </c>
+      <c r="C125" s="132"/>
+      <c r="D125" s="12"/>
+    </row>
+    <row r="126" s="133" customFormat="1" ht="33" customHeight="1">
+      <c r="A126" s="134" t="s">
+        <v>196</v>
+      </c>
+      <c r="B126" s="89" t="s">
+        <v>248</v>
+      </c>
+      <c r="C126" s="90"/>
+    </row>
+    <row r="127" s="12" customFormat="1" ht="28" customHeight="1">
+      <c r="A127" s="51">
         <v>0.67708333333333337</v>
       </c>
-      <c r="B124" s="118" t="s">
-        <v>197</v>
-      </c>
-      <c r="C124" s="118"/>
-      <c r="D124" s="12"/>
+      <c r="B127" s="136" t="s">
+        <v>199</v>
+      </c>
+      <c r="C127" s="136"/>
+      <c r="D127" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="45">
+  <mergeCells count="48">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="B6:C6"/>
@@ -4507,42 +4809,45 @@
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B24:C24"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="B37:C37"/>
     <mergeCell ref="B43:C43"/>
     <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
     <mergeCell ref="B52:C52"/>
     <mergeCell ref="A53:C53"/>
     <mergeCell ref="B54:C54"/>
     <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="A57:A59"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="A58:A60"/>
     <mergeCell ref="A64:A67"/>
     <mergeCell ref="A69:C69"/>
     <mergeCell ref="A70:C70"/>
     <mergeCell ref="A71:C71"/>
     <mergeCell ref="A73:C73"/>
     <mergeCell ref="B75:C75"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B88:C88"/>
-    <mergeCell ref="A89:A92"/>
-    <mergeCell ref="B89:C89"/>
-    <mergeCell ref="B95:C95"/>
+    <mergeCell ref="A76:C76"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="A87:C87"/>
+    <mergeCell ref="B90:C90"/>
+    <mergeCell ref="A91:A94"/>
+    <mergeCell ref="B91:C91"/>
     <mergeCell ref="B97:C97"/>
-    <mergeCell ref="A98:C98"/>
+    <mergeCell ref="B99:C99"/>
     <mergeCell ref="A100:C100"/>
-    <mergeCell ref="B101:C101"/>
-    <mergeCell ref="B102:C102"/>
+    <mergeCell ref="A102:C102"/>
     <mergeCell ref="B103:C103"/>
-    <mergeCell ref="B110:C110"/>
-    <mergeCell ref="B116:C116"/>
-    <mergeCell ref="B117:C117"/>
-    <mergeCell ref="B122:C122"/>
-    <mergeCell ref="B123:C123"/>
-    <mergeCell ref="B124:C124"/>
+    <mergeCell ref="B104:C104"/>
+    <mergeCell ref="B105:C105"/>
+    <mergeCell ref="A109:C109"/>
+    <mergeCell ref="B112:C112"/>
+    <mergeCell ref="B118:C118"/>
+    <mergeCell ref="B120:C120"/>
+    <mergeCell ref="B125:C125"/>
+    <mergeCell ref="B126:C126"/>
+    <mergeCell ref="B127:C127"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.51181102362204722" right="0.11811023622047245" top="0" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -4551,7 +4856,7 @@
   <rowBreaks count="3" manualBreakCount="3">
     <brk id="32" man="1" max="2"/>
     <brk id="70" man="1" max="2"/>
-    <brk id="97" man="1" max="2"/>
+    <brk id="99" man="1" max="2"/>
   </rowBreaks>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>